<commit_message>
Remove non-essential fields from Pathfactory Attend Live audit
Drop utm_id, Section 7 event tracking, and 21 Section 8 elements per
review. Keep core attendance, session engagement, and scoring fields.

Co-authored-by: demodolly <demodolly@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Pathfactory Events - Webinar Attend Live.xlsx
+++ b/Pathfactory Events - Webinar Attend Live.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q130"/>
+  <dimension ref="A1:Q106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4698,64 +4698,85 @@
       <c r="Q93" s="5" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>utm_id</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>Supports campaign instance-level attribution when multiple campaigns share naming.</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>Eloqua / Tealium</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Captured by Tealium from the attendance journey URL and passed to Eloqua with the Pathfactory payload when present.</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>N/A - captured by Tealium and passed to Eloqua when present</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L94" t="inlineStr"/>
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>8 - Activity Detail</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="n"/>
+      <c r="C94" s="4" t="n"/>
+      <c r="D94" s="4" t="n"/>
+      <c r="E94" s="4" t="n"/>
+      <c r="F94" s="4" t="n"/>
+      <c r="G94" s="4" t="n"/>
+      <c r="H94" s="4" t="n"/>
+      <c r="I94" s="4" t="n"/>
+      <c r="J94" s="4" t="n"/>
+      <c r="K94" s="4" t="n"/>
+      <c r="L94" s="4" t="n"/>
+      <c r="M94" s="4" t="n"/>
+      <c r="N94" s="4" t="n"/>
+      <c r="O94" s="4" t="n"/>
+      <c r="P94" s="4" t="n"/>
+      <c r="Q94" s="4" t="n"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>7 - Event Tracking Parameters</t>
-        </is>
-      </c>
+          <t>Attendance Date</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Timestamp for attribution sequencing, lead scoring recency, and operational reporting.</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Pathfactory / Eloqua</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Captured from Date Submitted on the Pathfactory attendance webhook payload in Eloqua.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>When was the attendance event submitted?</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Date/Time</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Event ID / EID</t>
+          <t>Event Time</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4765,7 +4786,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Links live attendance to the parent event for attribution and operational reporting.</t>
+          <t>Supports precise attendance timing for scoring and operational reporting.</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -4775,32 +4796,27 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Captured from EID on the Pathfactory attendance webhook payload in Eloqua.</t>
+          <t>Captured from Event Time on the Pathfactory attendance webhook payload.</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>What is the Event ID for this live virtual attendance?</t>
+          <t>What time did the attendance event occur?</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Time</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Potential</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
         <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>Potential</t>
         </is>
       </c>
       <c r="L96" t="inlineStr"/>
@@ -4808,7 +4824,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Event Name</t>
+          <t>Event Date</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4818,7 +4834,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Provides human-readable virtual event context for reporting and validation.</t>
+          <t>Supports event-day reporting and attribution alignment.</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -4828,68 +4844,98 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Captured from Virtual Event Name on the Pathfactory attendance webhook payload.</t>
+          <t>Captured from Event Date on the Pathfactory attendance webhook payload.</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>What is the name of the virtual event attended?</t>
+          <t>What date did the attendance event occur?</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Virtual Event Session Name</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Identifies the session attended for attribution and operational reporting.</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Pathfactory / Eloqua</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Captured from Virtual Event Session Name on the attendance webhook payload.</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Which virtual event session did the attendee join?</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="J97" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K97" t="inlineStr">
+      <c r="I98" t="inlineStr">
         <is>
           <t>Potential</t>
         </is>
       </c>
-      <c r="L97" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="4" t="inlineStr">
-        <is>
-          <t>8 - Activity Detail</t>
-        </is>
-      </c>
-      <c r="B98" s="4" t="n"/>
-      <c r="C98" s="4" t="n"/>
-      <c r="D98" s="4" t="n"/>
-      <c r="E98" s="4" t="n"/>
-      <c r="F98" s="4" t="n"/>
-      <c r="G98" s="4" t="n"/>
-      <c r="H98" s="4" t="n"/>
-      <c r="I98" s="4" t="n"/>
-      <c r="J98" s="4" t="n"/>
-      <c r="K98" s="4" t="n"/>
-      <c r="L98" s="4" t="n"/>
-      <c r="M98" s="4" t="n"/>
-      <c r="N98" s="4" t="n"/>
-      <c r="O98" s="4" t="n"/>
-      <c r="P98" s="4" t="n"/>
-      <c r="Q98" s="4" t="n"/>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Attendance Date</t>
+          <t>Virtual Event Session Slug</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Timestamp for attribution sequencing, lead scoring recency, and operational reporting.</t>
+          <t>URL-level session identifier for operational validation.</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -4899,41 +4945,30 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Captured from Date Submitted on the Pathfactory attendance webhook payload in Eloqua.</t>
+          <t>Captured from Virtual Event Session Slug on the attendance webhook payload.</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>When was the attendance event submitted?</t>
+          <t>What is the virtual event session slug?</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Date/Time</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K99" t="inlineStr">
-        <is>
           <t>Potential</t>
         </is>
       </c>
       <c r="L99" t="inlineStr"/>
-      <c r="M99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Webhook Name</t>
+          <t>Virtual Event Session Engagement Time (Minutes)</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4943,7 +4978,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Identifies the Pathfactory webhook integration for troubleshooting and operational audit.</t>
+          <t>Core engagement metric for lead scoring and content effectiveness on live attendance.</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -4953,17 +4988,22 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Captured from Webhook Name on the Pathfactory attendance payload.</t>
+          <t>Captured from Virtual Event Session Engagement Time (Minutes) on the attendance webhook payload.</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Which Pathfactory webhook delivered this attendance event?</t>
+          <t>How many minutes did the attendee engage with the live session?</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Text</t>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -4971,23 +5011,27 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Pathfactory Event Type</t>
+          <t>Visitor Registration Status (Session)</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Classifies the Pathfactory event for attribution models and activity routing.</t>
+          <t>Links attendance to session-level registration status for funnel analysis.</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -4997,12 +5041,12 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Captured from Event Type on the Pathfactory attendance webhook payload.</t>
+          <t>Captured from Visitor Registration Status (Session) on the attendance webhook payload.</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>What Pathfactory event type was recorded?</t>
+          <t>What is the visitor registration status for this session?</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -5017,31 +5061,25 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K101" t="inlineStr">
-        <is>
           <t>Potential</t>
         </is>
       </c>
       <c r="L101" t="inlineStr"/>
-      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Event Time</t>
+          <t>Visitor Registration Status (Event)</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Supports precise attendance timing for scoring and operational reporting.</t>
+          <t>Links attendance to event-level registration status for funnel analysis.</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5051,17 +5089,17 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Captured from Event Time on the Pathfactory attendance webhook payload.</t>
+          <t>Captured from Visitor Registration Status (Event) on the attendance webhook payload.</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>What time did the attendance event occur?</t>
+          <t>What is the visitor registration status for the event?</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -5071,16 +5109,15 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Potential</t>
         </is>
       </c>
       <c r="L102" t="inlineStr"/>
-      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Event Date</t>
+          <t>Pathfactory Session ID</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5090,7 +5127,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Supports event-day reporting and attribution alignment.</t>
+          <t>Session identifier from Pathfactory for deduplication and event stitching.</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -5100,17 +5137,17 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Captured from Event Date on the Pathfactory attendance webhook payload.</t>
+          <t>Captured from Session ID on the attendance webhook payload.</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>What date did the attendance event occur?</t>
+          <t>What is the Pathfactory session ID for this attendance?</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -5124,12 +5161,11 @@
         </is>
       </c>
       <c r="L103" t="inlineStr"/>
-      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Virtual Event Experience ID</t>
+          <t>Pathfactory Activity Type</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -5139,7 +5175,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Unique Pathfactory virtual event identifier for deduplication and taxonomy alignment.</t>
+          <t>Pathfactory activity classification for attribution and operational reporting.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -5149,12 +5185,12 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Captured from Virtual Event Experience ID on the attendance webhook payload.</t>
+          <t>Captured from activity_type on the attendance webhook payload.</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>What is the Virtual Event Experience ID?</t>
+          <t>What is the Pathfactory activity type?</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -5172,13 +5208,17 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
       <c r="L104" t="inlineStr"/>
-      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Virtual Event URL Slug</t>
+          <t>Primary Video Time Threshold Met</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -5188,7 +5228,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Links attendance to the published virtual event URL for operational validation.</t>
+          <t>Threshold-based engagement signal for lead scoring on video content within the event.</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -5198,12 +5238,12 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Captured from Virtual Event URL Slug on the attendance webhook payload.</t>
+          <t>Captured from Primary Video - Time Threshold Met on the attendance webhook payload.</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>What is the virtual event URL slug?</t>
+          <t>Which primary video time thresholds were met?</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -5211,28 +5251,32 @@
           <t>Text</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr">
+      <c r="I105" t="inlineStr">
         <is>
           <t>Potential</t>
         </is>
       </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
       <c r="L105" t="inlineStr"/>
-      <c r="M105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Virtual Event Start Time</t>
+          <t>Contact Source Original</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Supports scheduling alignment between registration and live attendance reporting.</t>
+          <t>Preserves original contact source for attribution lineage on attendance records.</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -5242,1187 +5286,30 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Captured from Virtual Event Start Time on the attendance webhook payload.</t>
+          <t>Captured from Contact Source Original on the attendance webhook payload when present.</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>When does the virtual event start?</t>
+          <t>What was the original contact source?</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Date/Time</t>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Potential</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K106" t="inlineStr">
-        <is>
           <t>Potential</t>
         </is>
       </c>
       <c r="L106" t="inlineStr"/>
-      <c r="M106" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>Virtual Event External ID 1</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>External reference for cross-system event alignment and reporting.</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>Captured from Virtual Event External ID 1 when present on the attendance payload.</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>What is Virtual Event External ID 1?</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="J107" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L107" t="inlineStr"/>
-      <c r="M107" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>Virtual Event External ID 2</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>Additional external reference for event alignment across systems.</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Captured from Virtual Event External ID 2 when present on the attendance payload.</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>What is Virtual Event External ID 2?</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="J108" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L108" t="inlineStr"/>
-      <c r="M108" t="inlineStr"/>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>Virtual Event External ID 3</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>Additional external reference for event alignment across systems.</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>Captured from Virtual Event External ID 3 when present on the attendance payload.</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>What is Virtual Event External ID 3?</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="J109" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L109" t="inlineStr"/>
-      <c r="M109" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>Virtual Event Session Name</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>Identifies the session attended for attribution and operational reporting.</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>Captured from Virtual Event Session Name on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>Which virtual event session did the attendee join?</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="J110" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K110" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L110" t="inlineStr"/>
-      <c r="M110" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>Virtual Event Session Slug</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>URL-level session identifier for operational validation.</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>Captured from Virtual Event Session Slug on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>What is the virtual event session slug?</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="J111" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L111" t="inlineStr"/>
-      <c r="M111" t="inlineStr"/>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>Virtual Event Session Start Time</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>Session-level scheduling for attendance validation and reporting.</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>Captured from Virtual Event Session Start Time on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>When does this session start?</t>
-        </is>
-      </c>
-      <c r="G112" t="inlineStr">
-        <is>
-          <t>Date/Time</t>
-        </is>
-      </c>
-      <c r="J112" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L112" t="inlineStr"/>
-      <c r="M112" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>Virtual Event Session External ID</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>External session identifier for deduplication and cross-system alignment.</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>Captured from Virtual Event Session External ID on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>What is the virtual event session external ID?</t>
-        </is>
-      </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="J113" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L113" t="inlineStr"/>
-      <c r="M113" t="inlineStr"/>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>Virtual Event Session Type</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>Distinguishes live, simulive, and related session types for scoring and reporting.</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Captured from Virtual Event Session Type on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>What type of virtual event session is this?</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>Picklist/Text</t>
-        </is>
-      </c>
-      <c r="I114" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="J114" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K114" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L114" t="inlineStr"/>
-      <c r="M114" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>Virtual Event Session Status</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>Confirms session state at time of attendance for operational quality checks.</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>Captured from Virtual Event Session Status on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>What is the session status when attendance was recorded?</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="J115" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L115" t="inlineStr"/>
-      <c r="M115" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Virtual Event Session Engagement Time (Minutes)</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>Core engagement metric for lead scoring and content effectiveness on live attendance.</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>Captured from Virtual Event Session Engagement Time (Minutes) on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>How many minutes did the attendee engage with the live session?</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="I116" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="J116" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K116" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L116" t="inlineStr"/>
-      <c r="M116" t="inlineStr"/>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>Visitor Registration Status (Session)</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>Links attendance to session-level registration status for funnel analysis.</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>Captured from Visitor Registration Status (Session) on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>What is the visitor registration status for this session?</t>
-        </is>
-      </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="J117" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L117" t="inlineStr"/>
-      <c r="M117" t="inlineStr"/>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>Visitor Registration Status (Event)</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>Links attendance to event-level registration status for funnel analysis.</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>Captured from Visitor Registration Status (Event) on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>What is the visitor registration status for the event?</t>
-        </is>
-      </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I118" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="J118" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L118" t="inlineStr"/>
-      <c r="M118" t="inlineStr"/>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>Content Journey</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>Captures Pathfactory content journey context for attribution analysis.</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>Captured from Content Journey on the attendance webhook payload when present.</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>What content journey preceded this live attendance?</t>
-        </is>
-      </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I119" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="K119" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L119" t="inlineStr"/>
-      <c r="M119" t="inlineStr"/>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>Supplemental Content Engagement</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>Indicates whether supplemental content was engaged during or around the session.</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Captured from Supplemental Content Engagement on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>Did the attendee engage with supplemental content?</t>
-        </is>
-      </c>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>Picklist/Text</t>
-        </is>
-      </c>
-      <c r="J120" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="K120" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L120" t="inlineStr"/>
-      <c r="M120" t="inlineStr"/>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>Supplemental Content Time Thresholds Met</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>Supports threshold-based scoring for supplemental content engagement.</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>Captured from Supplemental Content Time Thresholds Met on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>Which supplemental content time thresholds were met?</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="K121" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L121" t="inlineStr"/>
-      <c r="M121" t="inlineStr"/>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>Supplemental Content Engagement Time (Seconds)</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>Measures supplemental content depth for lead scoring beyond live session minutes.</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>Captured from Supplemental Content Engagement Time (Seconds) on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>How long did the attendee engage with supplemental content (seconds)?</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="J122" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="K122" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L122" t="inlineStr"/>
-      <c r="M122" t="inlineStr"/>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>Pathfactory Session ID</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>Session identifier from Pathfactory for deduplication and event stitching.</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>Captured from Session ID on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>What is the Pathfactory session ID for this attendance?</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I123" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="J123" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L123" t="inlineStr"/>
-      <c r="M123" t="inlineStr"/>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>Team</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>Operational routing or reporting metadata from Pathfactory when populated.</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>Captured from team on the attendance webhook payload when present.</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>What team value is associated with this attendance event?</t>
-        </is>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L124" t="inlineStr"/>
-      <c r="M124" t="inlineStr"/>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>Common Campaign ID</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Cross-system campaign alignment from Pathfactory attendance payload.</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>Captured from CCID on the attendance webhook payload when present.</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>What is the Common Campaign ID (CCID)?</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="J125" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L125" t="inlineStr"/>
-      <c r="M125" t="inlineStr"/>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>Conversica Flag</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>Indicates Conversica routing eligibility or processing from Pathfactory metadata.</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>Captured from conversica on the attendance webhook payload when present.</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>Is this attendance flagged for Conversica processing?</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>Picklist/Text</t>
-        </is>
-      </c>
-      <c r="J126" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L126" t="inlineStr"/>
-      <c r="M126" t="inlineStr"/>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>Pathfactory Activity Type</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>Pathfactory activity classification for attribution and operational reporting.</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>Captured from activity_type on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>What is the Pathfactory activity type?</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="J127" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K127" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L127" t="inlineStr"/>
-      <c r="M127" t="inlineStr"/>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>Pathfactory Asset Type</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>Classifies the Pathfactory asset associated with attendance for content reporting.</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>Captured from asset_type on the attendance webhook payload when present.</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>What Pathfactory asset type is associated with this attendance?</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="J128" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L128" t="inlineStr"/>
-      <c r="M128" t="inlineStr"/>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>Primary Video Time Threshold Met</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>Threshold-based engagement signal for lead scoring on video content within the event.</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>Captured from Primary Video - Time Threshold Met on the attendance webhook payload.</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>Which primary video time thresholds were met?</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L129" t="inlineStr"/>
-      <c r="M129" t="inlineStr"/>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>Contact Source Original</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>Preserves original contact source for attribution lineage on attendance records.</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>Pathfactory / Eloqua</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>Captured from Contact Source Original on the attendance webhook payload when present.</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>What was the original contact source?</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="J130" t="inlineStr">
-        <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="L130" t="inlineStr"/>
-      <c r="M130" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>